<commit_message>
Convert True/False category to Yes/No and add per-question images
- Statements file now uses Yes/No options (Yes=true, No=false); renamed to
  AZ-900_Kahoot_YesNo.xlsx (removed AZ-900_Kahoot_TrueFalse.xlsx)
- Updated Reference workbook (Yes-No sheet + README)
- Generated 36 subject-area images at kahoot_images/YesNo/YesNo_Qnn.png
- Added Yes-No sheet to the image guide; added .gitignore for __pycache__
</commit_message>
<xml_diff>
--- a/AZ-900_Kahoot_Image_Guide.xlsx
+++ b/AZ-900_Kahoot_Image_Guide.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Part 3" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Part 4" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Part 5" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Yes-No" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -453,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B14"/>
+  <dimension ref="B1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="116" customWidth="1" min="2" max="2"/>
@@ -538,6 +539,23 @@
       <c r="B14" t="inlineStr">
         <is>
           <t>without revealing the answer on screen. Images are generated (no third-party photos = no licensing issues).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>The 'Yes/No' sheet covers the Yes/No category (AZ-900_Kahoot_YesNo.xlsx); its images live in</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo and are named YesNo_Qnn.png in the same order as that file.</t>
         </is>
       </c>
     </row>
@@ -6883,4 +6901,1138 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Q #</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Statement</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Answer (Yes/No)</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Subject area</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Image file to drag in</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Kahoot image search keyword</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>You can create custom Azure roles to control access to resources.</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Identity &amp; Access</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q01.png</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>login security</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>A user account can be assigned to multiple Azure roles.</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Identity &amp; Access</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q02.png</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>login security</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>A resource group can have the Owner role assigned to multiple users.</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Identity &amp; Access</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q03.png</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>login security</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>An Azure subscription can have multiple account administrators.</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Cost &amp; Pricing</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q04.png</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>money budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>An Azure subscription can be managed by using a Microsoft account only.</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Cost &amp; Pricing</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q05.png</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>money budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>An Azure resource group can contain multiple Azure subscriptions.</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Cost &amp; Pricing</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q06.png</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>money budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Single sign-on requires all users to sign in with Microsoft Authenticator.</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Identity &amp; Access</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q07.png</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>login security</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Authentication establishes which level of access an authenticated user has.</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Identity &amp; Access</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q08.png</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>login security</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Conditional Access uses sign-in signals to allow or deny access.</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Identity &amp; Access</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q09.png</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>login security</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Data in an Azure Storage account automatically has at least three copies.</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q10.png</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>cloud data storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>All data in an Azure Storage account is auto-backed up to another datacenter.</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q11.png</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>cloud data storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>An Azure Storage account can hold only up to 2 TB and one million files.</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q12.png</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>cloud data storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Azure Reservations cost less than pay-as-you-go pricing.</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Cost &amp; Pricing</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q13.png</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>money budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Two Azure VMs of the same size always have the same monthly cost.</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Cost &amp; Pricing</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q14.png</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>money budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>When an Azure virtual machine is stopped, storage costs still apply.</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Cost &amp; Pricing</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q15.png</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>money budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Azure Files is an example of Infrastructure as a Service (IaaS).</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q16.png</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>cloud data storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>A DNS server on an Azure VM is an example of Platform as a Service (PaaS).</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Networking</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q17.png</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>computer network</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Microsoft Intune is an example of Software as a Service (SaaS).</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Cloud Concepts</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q18.png</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>cloud computing</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Creating and configuring a virtual network is part of the PaaS model.</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Networking</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q19.png</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>computer network</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Updating application code in Azure App Service is the customer's job.</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Compute</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q20.png</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>server computer</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Configuring user access in PaaS is the customer's responsibility.</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Cloud Concepts</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q21.png</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>cloud computing</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>A resource lock can be applied to a Microsoft Entra user.</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Identity &amp; Access</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q22.png</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>login security</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Multiple resource locks can be applied to the same virtual machine.</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Governance &amp; Mgmt</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q23.png</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>settings management</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>A delete lock allows modifying a resource but prevents deletion.</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Governance &amp; Mgmt</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q24.png</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>settings management</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Azure PowerShell can be installed on macOS.</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Governance &amp; Mgmt</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q25.png</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>settings management</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Azure Cloud Shell can be accessed from a Linux computer using a browser.</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Governance &amp; Mgmt</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q26.png</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>settings management</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>The Azure portal can be accessed only from Windows devices.</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Cloud Concepts</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q27.png</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>cloud computing</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Inbound traffic to Azure using ExpressRoute is always free.</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Networking</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q28.png</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>computer network</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Outbound traffic from Azure to on-premises networks is always free.</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Cloud Concepts</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q29.png</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>cloud computing</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Data transfer between Azure services in the same region is always free.</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Cloud Concepts</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q30.png</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>cloud computing</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Azure Monitor can monitor the performance of on-premises computers.</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Governance &amp; Mgmt</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q31.png</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>settings management</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Azure Monitor can send alerts to Microsoft Entra security groups.</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Identity &amp; Access</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q32.png</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>login security</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Azure Monitor can trigger alerts based on Log Analytics data.</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Governance &amp; Mgmt</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q33.png</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>settings management</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Only one tag can be assigned to an Azure resource.</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Governance &amp; Mgmt</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q34.png</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>settings management</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Tags can be assigned to resources using ARM templates.</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Governance &amp; Mgmt</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q35.png</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>settings management</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Tags can be used to enforce naming standards.</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Cloud Concepts</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>kahoot_images/YesNo/YesNo_Q36.png</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>cloud computing</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>